<commit_message>
Add LinkedIn URLs for 26 contacts
Colonne linkedin_url ajoutée au CSV/XLSX avec les profils LinkedIn
identifiés pour les DG, DRH et Responsables Formation/RH.

https://claude.ai/code/session_01FxoqYMicUtCHFPzbgaXBCv
</commit_message>
<xml_diff>
--- a/bailleurs_contacts.xlsx
+++ b/bailleurs_contacts.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +28,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -55,11 +59,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,11 +430,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K111"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
@@ -438,7 +443,8 @@
     <col width="42" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,6 +500,11 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>linkedin_url</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>source_url</t>
         </is>
       </c>
@@ -541,7 +552,12 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/posts/paris-habitat_cécile-belard-du-plantys-nouvelle-directrice-activity-6900366200384159744-f5z2</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -586,7 +602,12 @@
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/christopheargouddrh</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -632,6 +653,7 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -676,7 +698,12 @@
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/severine-leplus-095b0944</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -722,6 +749,7 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -767,6 +795,7 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -812,6 +841,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -857,6 +887,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -902,6 +933,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -947,6 +979,7 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -992,6 +1025,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1036,7 +1070,12 @@
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/isabelle-scapin-28964265</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1082,6 +1121,7 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1091,7 +1131,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Grenoble Alpes Métropole Habitat</t>
+          <t>Alpes Isère Habitat</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1106,15 +1146,28 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.grenoble-habitat.fr</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+          <t>https://alpeshabitat.fr</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Laurent</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Droulez</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Directeur Général</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1144,22 +1197,27 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Laurent</t>
+          <t>Cécile</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Droulez</t>
+          <t>May</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Directeur Général</t>
+          <t>Responsable Formation</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/c%C3%A9cile-may-84b57690/</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1169,42 +1227,43 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alpes Isère Habitat</t>
+          <t>OPAC Savoie</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Chambéry</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>73</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://alpeshabitat.fr</t>
+          <t>https://www.opac-savoie.fr</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Cécile</t>
+          <t>David</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Jonnard</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Responsable Formation</t>
+          <t>Directeur Général</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1214,32 +1273,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>OPAC Savoie</t>
+          <t>Toulouse Métropole Habitat</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Chambéry</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>31</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.opac-savoie.fr</t>
+          <t>https://www.toulouse-metropole-habitat.fr</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Luc</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Jonnard</t>
+          <t>Laventure</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1249,7 +1308,12 @@
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/luc-laventure-a16554195/</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1259,32 +1323,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Toulouse Métropole Habitat</t>
+          <t>Marseille Habitat</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.toulouse-metropole-habitat.fr</t>
+          <t>https://www.marseillehabitat.fr</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Luc</t>
+          <t>Frédéric</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Laventure</t>
+          <t>Pâris</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1295,6 +1359,7 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1304,7 +1369,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Marseille Habitat</t>
+          <t>Provence Métropole Logement (ex HMP)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1319,17 +1384,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.marseillehabitat.fr</t>
+          <t>https://www.habitat-marseille-provence.fr</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Frédéric</t>
+          <t>Jean-Bernard</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Pâris</t>
+          <t>Dambier</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1339,7 +1404,12 @@
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jean-bernard-dambier-44536b148/</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1349,32 +1419,32 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Provence Métropole Logement (ex Habitat Marseille Provence)</t>
+          <t>Var Habitat</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Toulon</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>83</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.habitat-marseille-provence.fr</t>
+          <t>https://www.varhabitat.com</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Jean-Bernard</t>
+          <t>Martial</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Dambier</t>
+          <t>Aubry</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1385,6 +1455,7 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1394,32 +1465,32 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Var Habitat</t>
+          <t>Gironde Habitat</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Toulon</t>
+          <t>Bordeaux</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>33</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.varhabitat.com</t>
+          <t>https://www.gironde-habitat.fr</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Martial</t>
+          <t>Sigrid</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Aubry</t>
+          <t>Monnier</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1429,7 +1500,12 @@
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/sigrid-monnier-62b45a24</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1439,7 +1515,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Gironde Habitat</t>
+          <t>Aquitanis (OPH Bordeaux Métropole)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1454,17 +1530,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.gironde-habitat.fr</t>
+          <t>https://www.aquitanis.fr</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sigrid</t>
+          <t>Jean-Luc</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Monnier</t>
+          <t>Gorce</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1475,6 +1551,7 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1484,32 +1561,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aquitanis (OPH Bordeaux Métropole)</t>
+          <t>Vendée Habitat</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>La Roche-sur-Yon</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>85</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.aquitanis.fr</t>
+          <t>https://www.vendeehabitat.fr</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Jean-Luc</t>
+          <t>Laurent</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Gorce</t>
+          <t>Saussaye</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1519,7 +1596,12 @@
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/laurent-saussaye-86118513a</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1529,22 +1611,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Vendée Habitat</t>
+          <t>Angers Loire Habitat</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>La Roche-sur-Yon</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>49</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.vendeehabitat.fr</t>
+          <t>https://www.angers-loire-habitat.fr</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1554,7 +1636,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Saussaye</t>
+          <t>Bordas</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1565,6 +1647,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1574,32 +1657,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Angers Loire Habitat</t>
+          <t>Archipel Habitat (OPH Rennes Métropole)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>35</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.angers-loire-habitat.fr</t>
+          <t>https://www.archipel-habitat.fr</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Laurent</t>
+          <t>Antoine</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Bordas</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1609,7 +1692,12 @@
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>https://rocketreach.co/antoine-rousseau-email_67702980</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1619,32 +1707,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Archipel Habitat (OPH Rennes Métropole)</t>
+          <t>Partenord Habitat</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Villeneuve d'Ascq</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>59</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.archipel-habitat.fr</t>
+          <t>https://www.partenordhabitat.fr</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Antoine</t>
+          <t>Eric</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Rousseau</t>
+          <t>Cojon</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1654,7 +1742,12 @@
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/eric-cojon-95a382181</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1684,22 +1777,27 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Eric</t>
+          <t>Matthieu</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Cojon</t>
+          <t>Canda</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Directeur Général</t>
+          <t>DRH</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/matthieu-canda-4aa78853/</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1709,12 +1807,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Partenord Habitat</t>
+          <t>Lille Métropole Habitat</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Villeneuve d'Ascq</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1724,27 +1822,28 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.partenordhabitat.fr</t>
+          <t>https://www.lmh.fr</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Matthieu</t>
+          <t>Emilie</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Canda</t>
+          <t>Lainard (Hakme)</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>DRH</t>
+          <t>Directeur Général</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1754,32 +1853,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Lille Métropole Habitat</t>
+          <t>Pas-de-Calais Habitat</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Arras</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>62</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.lmh.fr</t>
+          <t>https://www.pasdecalais-habitat.fr</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Emilie</t>
+          <t>Bruno</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Lainard (Hakme)</t>
+          <t>Fontalirand</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1790,6 +1889,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1799,32 +1899,32 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Pas-de-Calais Habitat</t>
+          <t>Habitat 76</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Arras</t>
+          <t>Rouen</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>76</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.pasdecalais-habitat.fr</t>
+          <t>https://habitat76.fr</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Bruno</t>
+          <t>Eric</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Fontalirand</t>
+          <t>Gimer</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1835,6 +1935,7 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1844,32 +1945,32 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Habitat 76</t>
+          <t>Inolya (OPH Calvados)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Rouen</t>
+          <t>Caen</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://habitat76.fr</t>
+          <t>https://www.inolya.fr</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Eric</t>
+          <t>Christophe</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Gimer</t>
+          <t>Bureau</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1880,6 +1981,7 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1889,32 +1991,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Inolya (OPH Calvados)</t>
+          <t>Meurthe-et-Moselle Habitat (MMH)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Caen</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>54</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.inolya.fr</t>
+          <t>https://www.mmhabitat.fr</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Christophe</t>
+          <t>Audrey</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Bureau</t>
+          <t>Dony</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1925,6 +2027,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1934,32 +2037,32 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Meurthe-et-Moselle Habitat (MMH)</t>
+          <t>Vosgelis</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Épinal</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>88</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.mmhabitat.fr</t>
+          <t>https://www.vosgelis.fr</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Audrey</t>
+          <t>Fabrice</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Dony</t>
+          <t>Barbe</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1969,7 +2072,12 @@
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/fabrice-barbe</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1999,22 +2107,23 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Fabrice</t>
+          <t>Lorinda</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Barbe</t>
+          <t>Carreiras</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Directeur Général</t>
+          <t>DRH</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2024,42 +2133,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Vosgelis</t>
+          <t>Orvitis</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Épinal</t>
+          <t>Dijon</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.vosgelis.fr</t>
+          <t>https://www.orvitis.fr</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Lorinda</t>
+          <t>Christophe</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Carreiras</t>
+          <t>Bérion</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>DRH</t>
+          <t>Directeur Général</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/christophe-berion-76611558</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2089,22 +2203,27 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Christophe</t>
+          <t>Josiane</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Bérion</t>
+          <t>Corte</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Directeur Général</t>
+          <t>DRH</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/josiane-corte-87108090</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2114,42 +2233,43 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Orvitis</t>
+          <t>Dynacité</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Dijon</t>
+          <t>Oyonnax</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.orvitis.fr</t>
+          <t>https://www.dynacite.fr</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Josiane</t>
+          <t>Jean-Luc</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Corte</t>
+          <t>Triollet</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>DRH</t>
+          <t>Directeur Général</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2179,22 +2299,23 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Jean-Luc</t>
+          <t>Nathalie</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Triollet</t>
+          <t>Marotta</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Directeur Général</t>
+          <t>DRH</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2204,42 +2325,43 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Dynacité</t>
+          <t>Allier Habitat</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Oyonnax</t>
+          <t>Moulins</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>03</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.dynacite.fr</t>
+          <t>https://www.allier-habitat.fr</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Nathalie</t>
+          <t>Laurent</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Marotta</t>
+          <t>Cot</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>DRH</t>
+          <t>Directeur Général</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2249,32 +2371,32 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Allier Habitat</t>
+          <t>Hérault Logement</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Moulins</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://www.allier-habitat.fr</t>
+          <t>https://www.herault-logement.fr</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Laurent</t>
+          <t>Gilles</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Cot</t>
+          <t>Dupont</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2285,6 +2407,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2294,42 +2417,31 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Hérault Logement</t>
+          <t>Nantes Métropole Habitat</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Montpellier</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>44</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.herault-logement.fr</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Gilles</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Dupont</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Directeur Général</t>
-        </is>
-      </c>
+          <t>https://www.nmh.fr</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2339,22 +2451,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Nantes Métropole Habitat</t>
+          <t>Saône-et-Loire Habitat</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Mâcon</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>71</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.nmh.fr</t>
+          <t>https://www.sl-habitat.fr</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -2363,6 +2475,7 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2372,22 +2485,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Saône-et-Loire Habitat</t>
+          <t>Yvelines Habitat</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Mâcon</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>78</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.sl-habitat.fr</t>
+          <t>https://www.yvelineshabitat.fr</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2396,6 +2509,7 @@
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2405,22 +2519,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Yvelines Habitat</t>
+          <t>Seine-et-Marne Habitat</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Versailles</t>
+          <t>Dammarie-les-Lys</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>77</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://www.yvelineshabitat.fr</t>
+          <t>https://www.seineetmarnehabitat.fr</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2429,6 +2543,7 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2438,22 +2553,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Seine-et-Marne Habitat</t>
+          <t>Côte-d'Or Habitat</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Dammarie-les-Lys</t>
+          <t>Dijon</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://www.seineetmarnehabitat.fr</t>
+          <t>https://www.cotedorhabitat.fr</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -2462,6 +2577,7 @@
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2471,22 +2587,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Côte-d'Or Habitat</t>
+          <t>Haute-Loire Habitat</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Dijon</t>
+          <t>Le Puy-en-Velay</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>43</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.cotedorhabitat.fr</t>
+          <t>https://www.hauteloirehabitat.fr</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -2495,6 +2611,7 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2504,22 +2621,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Haute-Loire Habitat</t>
+          <t>Puy-de-Dôme Habitat</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Le Puy-en-Velay</t>
+          <t>Clermont-Ferrand</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>63</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.hauteloirehabitat.fr</t>
+          <t>https://www.puy-de-dome-habitat.fr</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2528,6 +2645,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2537,22 +2655,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Puy-de-Dôme Habitat</t>
+          <t>Moselle Habitat</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Clermont-Ferrand</t>
+          <t>Metz</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>57</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.puy-de-dome-habitat.fr</t>
+          <t>https://www.mosellehabitat.fr</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2561,6 +2679,7 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2570,22 +2689,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Moselle Habitat</t>
+          <t>Bas-Rhin Habitat</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Metz</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>67</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://www.mosellehabitat.fr</t>
+          <t>https://www.basrhinhabitat.fr</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2594,6 +2713,7 @@
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2603,7 +2723,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Bas-Rhin Habitat</t>
+          <t>Alsace Habitat</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2618,7 +2738,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.basrhinhabitat.fr</t>
+          <t>https://www.alsacehabitat.fr</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2627,6 +2747,7 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2636,22 +2757,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alsace Habitat</t>
+          <t>Nord Habitat</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Strasbourg</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>59</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://www.alsacehabitat.fr</t>
+          <t>https://www.nordhabitat.fr</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -2660,6 +2781,7 @@
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2669,22 +2791,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Nord Habitat</t>
+          <t>Côtes d'Armor Habitat</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Saint-Brieuc</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://www.nordhabitat.fr</t>
+          <t>https://www.cotesdarmor-habitat.fr</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -2693,6 +2815,7 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2702,22 +2825,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Côtes d'Armor Habitat</t>
+          <t>Manche Habitat</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Saint-Brieuc</t>
+          <t>Saint-Lô</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://www.cotesdarmor-habitat.fr</t>
+          <t>https://www.manchehabitat.fr</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -2726,6 +2849,7 @@
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2735,22 +2859,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Manche Habitat</t>
+          <t>Morbihan Habitat (ex Bretagne Sud Habitat)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Saint-Lô</t>
+          <t>Vannes</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>56</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://www.manchehabitat.fr</t>
+          <t>https://www.morbihan-habitat.fr</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2759,6 +2883,7 @@
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2768,22 +2893,22 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Bretagne Sud Habitat / Morbihan Habitat</t>
+          <t>Bourgogne Habitat</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Vannes</t>
+          <t>Dijon</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://www.bretagne-sud-habitat.fr</t>
+          <t>https://www.bourgognehabitat.fr</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -2792,6 +2917,7 @@
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2801,22 +2927,22 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Bourgogne Habitat</t>
+          <t>Habitat 13</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Dijon</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://www.bourgognehabitat.fr</t>
+          <t>https://www.habitat13.fr</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -2825,6 +2951,7 @@
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2834,22 +2961,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Habitat 13</t>
+          <t>Nice Habitat</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Nice</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>06</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://www.habitat13.fr</t>
+          <t>https://www.nicehabitat.fr</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -2858,6 +2985,7 @@
       <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2867,22 +2995,22 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Nice Habitat</t>
+          <t>Deux Fleuves Loire Habitat (ex Loire Habitat)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Saint-Étienne</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://www.nicehabitat.fr</t>
+          <t>https://www.deuxfleuvesloirehabitat.fr</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
@@ -2891,39 +3019,53 @@
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>OPH</t>
+          <t>ESH</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Deux Fleuves Loire Habitat (ex Loire Habitat)</t>
+          <t>Immobilière 3F</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Saint-Étienne</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>75</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://www.rhonehabitat.fr</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+          <t>https://www.groupe3f.fr</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Valérie</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Fournier</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Directeur Général</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2958,17 +3100,22 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Fournier</t>
+          <t>Chung-Coquillet</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Directeur Général</t>
+          <t>DRH</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/val%C3%A9rie-chung-coquillet-2b2500121/</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2978,7 +3125,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Immobilière 3F</t>
+          <t>ICF Habitat</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2993,27 +3140,32 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://www.groupe3f.fr</t>
+          <t>https://www.icfhabitat.fr</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Valérie</t>
+          <t>Romain</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Chung-Coquillet</t>
+          <t>Dubois</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>DRH</t>
+          <t>Directeur Général</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/romain-dubois-26964521</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3043,22 +3195,27 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Romain</t>
+          <t>Valérie</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Dubois</t>
+          <t>Bignon</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Directeur Général</t>
+          <t>DRH</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/val%C3%A9rie-bignon-86ab9330</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3068,7 +3225,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ICF Habitat</t>
+          <t>RIVP</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3083,27 +3240,32 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://www.icfhabitat.fr</t>
+          <t>https://www.rivp.fr</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Valérie</t>
+          <t>Christine</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Bignon</t>
+          <t>Laconde</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>DRH</t>
+          <t>Directeur Général</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/christine-laconde-4452a0269</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3113,7 +3275,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>RIVP</t>
+          <t>Efidis (CDC Habitat Social)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3128,27 +3290,16 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://www.rivp.fr</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Christine</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>Laconde</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>Directeur Général</t>
-        </is>
-      </c>
+          <t>https://www.efidis.fr</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3158,7 +3309,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Efidis</t>
+          <t>Domaxis</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3173,15 +3324,28 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>https://www.efidis.fr</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
+          <t>https://www.domaxis.fr</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Bruno</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Hoang</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Directeur Général Adjoint</t>
+        </is>
+      </c>
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3211,22 +3375,27 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Bruno</t>
+          <t>Marie-Claude</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Hoang</t>
+          <t>Gauthier</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Directeur Général Adjoint</t>
+          <t>DRH</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/marie-claude-gauthier-03091436</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3236,42 +3405,43 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Domaxis</t>
+          <t>Vilogia</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Villeneuve d'Ascq</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>59</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>https://www.domaxis.fr</t>
+          <t>https://www.vilogia.fr</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Marie-Claude</t>
+          <t>Philippe</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Gauthier</t>
+          <t>Rémignon</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>DRH</t>
+          <t>Président Directoire</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3281,7 +3451,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Vilogia</t>
+          <t>Habitat du Nord</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3296,17 +3466,17 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://www.vilogia.fr</t>
+          <t>https://www.habitatdunord.fr</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Philippe</t>
+          <t>Franck</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Rémignon</t>
+          <t>Porier</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3317,6 +3487,7 @@
       <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3326,42 +3497,43 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Habitat du Nord</t>
+          <t>Batigère</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Villeneuve d'Ascq</t>
+          <t>Metz</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>57</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>https://www.habitatdunord.fr</t>
+          <t>https://www.batigere.fr</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Franck</t>
+          <t>Jean-François</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Porier</t>
+          <t>Prevot</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Président Directoire</t>
+          <t>Directeur Général Groupe</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3371,30 +3543,43 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Partenord Habitat</t>
+          <t>Batigère</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Villeneuve d'Ascq</t>
+          <t>Metz</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>57</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://www.partenord-legroupe.fr</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
+          <t>https://www.batigere.fr</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Nathalie</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Mateos-Jorge</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Directeur Général Adjoint Groupe</t>
+        </is>
+      </c>
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3424,22 +3609,23 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Jean-François</t>
+          <t>Sébastien</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Prevot</t>
+          <t>Tilignac</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Directeur Général Groupe</t>
+          <t>Directeur Général Batigère Grand Est</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3449,42 +3635,43 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Batigère</t>
+          <t>Néolia</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Metz</t>
+          <t>Besançon</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://www.batigere.fr</t>
+          <t>https://www.neolia.fr</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Nathalie</t>
+          <t>Jacques</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Mateos-Jorge</t>
+          <t>Ferrand</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Directeur Général Adjoint Groupe</t>
+          <t>Directeur Général</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3494,42 +3681,31 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Batigère</t>
+          <t>Alliade Habitat</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Metz</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://www.batigere.fr</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>Sébastien</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>Tilignac</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>Directeur Général Batigère Grand Est</t>
-        </is>
-      </c>
+          <t>https://alliadehabitat.com</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3539,32 +3715,32 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Néolia</t>
+          <t>Semcoda</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Besançon</t>
+          <t>Bourg-en-Bresse</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://www.neolia.fr</t>
+          <t>https://www.semcoda.com</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Jacques</t>
+          <t>Bernard</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Ferrand</t>
+          <t>Perret</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3574,7 +3750,12 @@
       </c>
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/bernard-perret-729057263/</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3584,42 +3765,47 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Alliade Habitat</t>
+          <t>Erilia</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>https://alliadehabitat.com</t>
+          <t>https://www.erilia.fr</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Frédéric</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Kada</t>
+          <t>Lavergne</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>RH Business Partner</t>
+          <t>Directeur Général</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/fr%C3%A9d%C3%A9ric-lavergne-5617508</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3629,42 +3815,47 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Semcoda</t>
+          <t>Erilia</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Bourg-en-Bresse</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>https://www.semcoda.com</t>
+          <t>https://www.erilia.fr</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Bernard</t>
+          <t>Fabienne</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Perret</t>
+          <t>Abecassis</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Directeur Général</t>
+          <t>Directeur Général Délégué</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/fabienne-abecassis-34b01830</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3674,30 +3865,43 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Dynacité (ESH)</t>
+          <t>Erilia</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Oyonnax</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>https://www.dynacite.fr</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
+          <t>https://www.erilia.fr</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Antoine</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Jeandet</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Directeur Général Délégué</t>
+        </is>
+      </c>
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3707,7 +3911,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Erilia</t>
+          <t>Logirem</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3722,17 +3926,17 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>https://www.erilia.fr</t>
+          <t>https://www.logirem.fr</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Frédéric</t>
+          <t>Fabienne</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Lavergne</t>
+          <t>Abecassis</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3742,7 +3946,12 @@
       </c>
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/fabienne-abecassis-34b01830</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3752,7 +3961,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Erilia</t>
+          <t>Logirem</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3767,17 +3976,17 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://www.erilia.fr</t>
+          <t>https://www.logirem.fr</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Fabienne</t>
+          <t>Frank</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Abecassis</t>
+          <t>Nicol</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3788,6 +3997,7 @@
       <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3797,42 +4007,43 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Erilia</t>
+          <t>Espacil Habitat</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>35</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://www.erilia.fr</t>
+          <t>https://www.espacil-habitat.fr</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Antoine</t>
+          <t>Julia</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Jeandet</t>
+          <t>Lagadec</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Directeur Général Délégué</t>
+          <t>Directeur Général</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3842,32 +4053,32 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Logirem</t>
+          <t>Aiguillon Construction</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>35</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://www.logirem.fr</t>
+          <t>https://www.aiguillon-construction.fr</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Fabienne</t>
+          <t>Thierry</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Abecassis</t>
+          <t>Heyvang</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3877,7 +4088,12 @@
       </c>
       <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/thierry-heyvang-b952bb26/</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3887,32 +4103,32 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Logirem</t>
+          <t>Aiguillon Construction</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>35</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://www.logirem.fr</t>
+          <t>https://www.aiguillon-construction.fr</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Frank</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Nicol</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -3923,6 +4139,7 @@
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3932,32 +4149,32 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Espacil Habitat</t>
+          <t>Harmonie Habitat</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Saint-Herblain</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>44</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>https://www.espacil-habitat.fr</t>
+          <t>https://www.harmoniehabitat.org</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Julia</t>
+          <t>Fabienne</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Lagadec</t>
+          <t>Delcambre</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -3967,7 +4184,12 @@
       </c>
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/fabienne-delcambre-38aab8145</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3977,42 +4199,43 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Aiguillon Construction</t>
+          <t>Harmonie Habitat</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Saint-Herblain</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>44</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>https://www.aiguillon-construction.fr</t>
+          <t>https://www.harmoniehabitat.org</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Thierry</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Heyvang</t>
+          <t>Riand</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Directeur Général</t>
+          <t>Directeur Général Adjoint – Ressources</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4022,42 +4245,31 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Aiguillon Construction</t>
+          <t>Clairsienne</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Bordeaux</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>33</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>https://www.aiguillon-construction.fr</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>Thomas</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>Duke</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>Directeur Général Délégué</t>
-        </is>
-      </c>
+          <t>https://www.clairsienne.com</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4067,42 +4279,31 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Harmonie Habitat</t>
+          <t>Nouveau Logis</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Saint-Herblain</t>
+          <t>Bordeaux</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>33</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://www.harmoniehabitat.org</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>Fabienne</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>Delcambre</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>Directeur Général</t>
-        </is>
-      </c>
+          <t>https://www.nouveaulogis.fr</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4112,42 +4313,31 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Harmonie Habitat</t>
+          <t>SCIC Habitat</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Saint-Herblain</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>75</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://www.harmoniehabitat.org</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>Helena</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>Riand</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>Directeur Général Adjoint – Ressources</t>
-        </is>
-      </c>
+          <t>https://www.scic-habitat.fr</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4157,22 +4347,22 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Clairsienne</t>
+          <t>France Habitation</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>75</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>https://www.clairsienne.com</t>
+          <t>https://www.france-habitation.fr</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4181,6 +4371,7 @@
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4190,22 +4381,22 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Nouveau Logis</t>
+          <t>OGIF</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>75</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://www.nouveaulogis.fr</t>
+          <t>https://www.ogif.fr</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4214,6 +4405,7 @@
       <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4223,22 +4415,22 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Vosgelis ESH</t>
+          <t>Logi-Ouest</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Épinal</t>
+          <t>Brest</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>29</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://www.vosgelis.fr</t>
+          <t>https://www.logiouest.fr</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4247,6 +4439,7 @@
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4256,22 +4449,22 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SCIC Habitat</t>
+          <t>Sarthe Habitat</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Le Mans</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>72</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://www.scic-habitat.fr</t>
+          <t>https://www.sarthehabitat.fr</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4280,6 +4473,7 @@
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4289,22 +4483,22 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>France Habitation</t>
+          <t>Picardie Habitat</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>https://www.france-habitation.fr</t>
+          <t>https://www.picardiehabitat.fr</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4313,6 +4507,7 @@
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr"/>
       <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4322,22 +4517,22 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>OGIF</t>
+          <t>Aisne Habitat</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Laon</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>02</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>https://www.ogif.fr</t>
+          <t>https://www.aisnehabitat.fr</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4346,6 +4541,7 @@
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4355,22 +4551,22 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Orvitis ESH</t>
+          <t>Habitat 62/59 Picardie</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Dijon</t>
+          <t>Arras</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>62</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>https://www.orvitis.fr</t>
+          <t>https://www.habitat6259picardie.fr</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4379,6 +4575,7 @@
       <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4388,22 +4585,22 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Logi-Ouest</t>
+          <t>Néodyme</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Brest</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>https://www.logiouest.fr</t>
+          <t>https://www.neodyme.org</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4412,6 +4609,7 @@
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4421,22 +4619,22 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Vendée Habitat ESH</t>
+          <t>Haute-Saône Habitat</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>La Roche-sur-Yon</t>
+          <t>Vesoul</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>70</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>https://www.vendeehabitat.fr</t>
+          <t>https://www.hsh70.fr</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4445,6 +4643,7 @@
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr"/>
       <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4454,22 +4653,22 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Sarthe Habitat</t>
+          <t>Nièvre Habitat</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Le Mans</t>
+          <t>Nevers</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>58</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>https://www.sarthehabitat.fr</t>
+          <t>https://www.nievre-habitat.com</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4478,6 +4677,7 @@
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4487,22 +4687,22 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Picardie Habitat</t>
+          <t>Cher Habitat</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Bourges</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://www.picardiehabitat.fr</t>
+          <t>https://www.cherhabitat.fr</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4511,6 +4711,7 @@
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4520,22 +4721,22 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Aisne Habitat</t>
+          <t>Indre Habitat</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Laon</t>
+          <t>Châteauroux</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>https://www.aisnehabitat.fr</t>
+          <t>https://www.indrehabitat.fr</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4544,6 +4745,7 @@
       <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4553,22 +4755,22 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Habitat 62/59 Picardie</t>
+          <t>Loir-et-Cher Habitat</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Arras</t>
+          <t>Blois</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>41</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://www.habitat6259picardie.fr</t>
+          <t>https://www.lchabitat.fr</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -4577,6 +4779,7 @@
       <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr"/>
       <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4586,22 +4789,22 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Néodyme</t>
+          <t>Loiret Habitat</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Orléans</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>45</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://www.neodyme.org</t>
+          <t>https://www.loirethabitat.fr</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4610,6 +4813,7 @@
       <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4619,22 +4823,22 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Habitat 80</t>
+          <t>Eure-et-Loir Habitat</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Amiens</t>
+          <t>Chartres</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>28</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>https://www.habitat80.fr</t>
+          <t>https://www.euretloir-habitat.fr</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -4643,6 +4847,7 @@
       <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr"/>
       <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4652,22 +4857,22 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Haute-Saône Habitat</t>
+          <t>Héritage et Traditions Habitat</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Vesoul</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>https://www.hsh70.fr</t>
+          <t>https://www.ht-habitat.fr</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -4676,6 +4881,7 @@
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4685,22 +4891,22 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Nièvre Habitat</t>
+          <t>Habitat 80</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Nevers</t>
+          <t>Amiens</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>https://www.nievre-habitat.com</t>
+          <t>https://www.habitat80.fr</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -4709,206 +4915,37 @@
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>ESH</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>Cher Habitat</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>Bourges</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>https://www.cherhabitat.fr</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>ESH</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Indre Habitat</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>Châteauroux</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>https://www.indrehabitat.fr</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>ESH</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>Loir-et-Cher Habitat</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>Blois</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>https://www.lchabitat.fr</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>ESH</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>Loiret Habitat</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>Orléans</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>https://www.loirethabitat.fr</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>ESH</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>Eure-et-Loir Habitat</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>Chartres</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>https://www.euretloir-habitat.fr</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>ESH</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Héritage et Traditions Habitat</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>Lyon</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>69</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>https://www.ht-habitat.fr</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId26"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add telephone_mobile column; confirm Christophe Argoud 06 46 19 07 56
- Add telephone_mobile field to FIELDNAMES, DATA tuples, and build_rows()
- Only one public 06/07 mobile found after exhaustive search: Christophe Argoud
  (DRH Paris Habitat) — 06 46 19 07 56, sourced from DoyouBuzz/Viadeo profiles
- All other executives' mobiles are behind paid enrichment paywalls (Lusha, Kaspr,
  Fullenrich, RocketReach) and not publicly indexed

https://claude.ai/code/session_01FxoqYMicUtCHFPzbgaXBCv
</commit_message>
<xml_diff>
--- a/bailleurs_contacts.xlsx
+++ b/bailleurs_contacts.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:M105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -443,8 +443,9 @@
     <col width="42" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,10 +501,15 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>telephone_mobile</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>linkedin_url</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
@@ -552,12 +558,13 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/posts/paris-habitat_cécile-belard-du-plantys-nouvelle-directrice-activity-6900366200384159744-f5z2</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -602,12 +609,17 @@
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>06 46 19 07 56</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/christopheargouddrh</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -654,6 +666,7 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -698,12 +711,13 @@
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/severine-leplus-095b0944</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -750,6 +764,7 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -796,6 +811,7 @@
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -842,6 +858,7 @@
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -888,6 +905,7 @@
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -934,6 +952,7 @@
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -980,6 +999,7 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1026,6 +1046,7 @@
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1070,12 +1091,13 @@
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/isabelle-scapin-28964265</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1122,6 +1144,7 @@
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1168,6 +1191,7 @@
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1212,12 +1236,13 @@
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/c%C3%A9cile-may-84b57690/</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1264,6 +1289,7 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1308,12 +1334,13 @@
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/luc-laventure-a16554195/</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1360,6 +1387,7 @@
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1404,12 +1432,13 @@
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/jean-bernard-dambier-44536b148/</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1456,6 +1485,7 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1500,12 +1530,13 @@
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/sigrid-monnier-62b45a24</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1552,6 +1583,7 @@
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1596,12 +1628,13 @@
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/laurent-saussaye-86118513a</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1648,6 +1681,7 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1692,12 +1726,13 @@
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>https://rocketreach.co/antoine-rousseau-email_67702980</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1742,12 +1777,13 @@
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/eric-cojon-95a382181</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1792,12 +1828,13 @@
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/matthieu-canda-4aa78853/</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1844,6 +1881,7 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1890,6 +1928,7 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1936,6 +1975,7 @@
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1982,6 +2022,7 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2028,6 +2069,7 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2072,12 +2114,13 @@
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/fabrice-barbe</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2124,6 +2167,7 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2168,12 +2212,13 @@
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/christophe-berion-76611558</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2218,12 +2263,13 @@
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/josiane-corte-87108090</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2270,6 +2316,7 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2316,6 +2363,7 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2362,6 +2410,7 @@
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2408,6 +2457,7 @@
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2442,6 +2492,7 @@
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2476,6 +2527,7 @@
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2510,6 +2562,7 @@
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2544,6 +2597,7 @@
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2578,6 +2632,7 @@
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2612,6 +2667,7 @@
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2646,6 +2702,7 @@
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2680,6 +2737,7 @@
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2714,6 +2772,7 @@
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2748,6 +2807,7 @@
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2782,6 +2842,7 @@
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2816,6 +2877,7 @@
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2850,6 +2912,7 @@
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2884,6 +2947,7 @@
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2918,6 +2982,7 @@
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2952,6 +3017,7 @@
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2986,6 +3052,7 @@
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3020,6 +3087,7 @@
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3066,6 +3134,7 @@
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3110,12 +3179,13 @@
       </c>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr"/>
-      <c r="K61" s="2" t="inlineStr">
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/val%C3%A9rie-chung-coquillet-2b2500121/</t>
         </is>
       </c>
-      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3160,12 +3230,13 @@
       </c>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr"/>
-      <c r="K62" s="2" t="inlineStr">
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/romain-dubois-26964521</t>
         </is>
       </c>
-      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3210,12 +3281,13 @@
       </c>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr"/>
-      <c r="K63" s="2" t="inlineStr">
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/val%C3%A9rie-bignon-86ab9330</t>
         </is>
       </c>
-      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3260,12 +3332,13 @@
       </c>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr"/>
-      <c r="K64" s="2" t="inlineStr">
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/christine-laconde-4452a0269</t>
         </is>
       </c>
-      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3300,6 +3373,7 @@
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3346,6 +3420,7 @@
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3390,12 +3465,13 @@
       </c>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr"/>
-      <c r="K67" s="2" t="inlineStr">
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/marie-claude-gauthier-03091436</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3442,6 +3518,7 @@
       <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3488,6 +3565,7 @@
       <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3534,6 +3612,7 @@
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3580,6 +3659,7 @@
       <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3626,6 +3706,7 @@
       <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3672,6 +3753,7 @@
       <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3706,6 +3788,7 @@
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3750,12 +3833,13 @@
       </c>
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr"/>
-      <c r="K75" s="2" t="inlineStr">
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" s="2" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/bernard-perret-729057263/</t>
         </is>
       </c>
-      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3800,12 +3884,13 @@
       </c>
       <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr"/>
-      <c r="K76" s="2" t="inlineStr">
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/fr%C3%A9d%C3%A9ric-lavergne-5617508</t>
         </is>
       </c>
-      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3850,12 +3935,13 @@
       </c>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr"/>
-      <c r="K77" s="2" t="inlineStr">
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/fabienne-abecassis-34b01830</t>
         </is>
       </c>
-      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3902,6 +3988,7 @@
       <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3946,12 +4033,13 @@
       </c>
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr"/>
-      <c r="K79" s="2" t="inlineStr">
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/fabienne-abecassis-34b01830</t>
         </is>
       </c>
-      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3998,6 +4086,7 @@
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4044,6 +4133,7 @@
       <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4088,12 +4178,13 @@
       </c>
       <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr"/>
-      <c r="K82" s="2" t="inlineStr">
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/thierry-heyvang-b952bb26/</t>
         </is>
       </c>
-      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4140,6 +4231,7 @@
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4184,12 +4276,13 @@
       </c>
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr"/>
-      <c r="K84" s="2" t="inlineStr">
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr">
         <is>
           <t>https://fr.linkedin.com/in/fabienne-delcambre-38aab8145</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4236,6 +4329,7 @@
       <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4270,6 +4364,7 @@
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4304,6 +4399,7 @@
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4338,6 +4434,7 @@
       <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4372,6 +4469,7 @@
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4406,6 +4504,7 @@
       <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4440,6 +4539,7 @@
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4474,6 +4574,7 @@
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4508,6 +4609,7 @@
       <c r="J93" t="inlineStr"/>
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4542,6 +4644,7 @@
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4576,6 +4679,7 @@
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4610,6 +4714,7 @@
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4644,6 +4749,7 @@
       <c r="J97" t="inlineStr"/>
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4678,6 +4784,7 @@
       <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4712,6 +4819,7 @@
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4746,6 +4854,7 @@
       <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4780,6 +4889,7 @@
       <c r="J101" t="inlineStr"/>
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4814,6 +4924,7 @@
       <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4848,6 +4959,7 @@
       <c r="J103" t="inlineStr"/>
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4882,6 +4994,7 @@
       <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4916,35 +5029,36 @@
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L61" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L62" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L63" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L64" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L75" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L76" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L77" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L79" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L82" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L84" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>